<commit_message>
Data templates: linear one-row-per-product BOM layout
- Replace long-form Assembly_BOM with linear (one row per product) sheets:
  Panel_BOM (board + face/back veneer + glue g/face + packing + optional uv_topcoat)
  and DoorSkin_BOM (board + primer pass1/pass2 g/m² + packing). Much easier to fill.
- Transform_PVS/PSP unchanged
</commit_message>
<xml_diff>
--- a/templates/pvwood_bom.xlsx
+++ b/templates/pvwood_bom.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assembly_BOM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Transform_PVS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Transform_PSP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Panel_BOM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DoorSkin_BOM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Transform_PVS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Transform_PSP" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -463,35 +464,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Assembly_BOM: one row per BOM line. role dropdown; use item_code OR glue_recipe_code.</t>
+          <t>ONE ROW PER PRODUCT — fill the component code into each column.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Main-line products: BOARD + FACE/BACK_VENEER + FACE/BACK_GLUE + PACKING.</t>
+          <t>Panel_BOM (main lines P01/P02/P37): board + face/back veneer + glue (g/face each</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PUV Mode-A door skins: BOARD + PRIMER (usage_g_per_m2, note pass1/pass2).</t>
+          <t xml:space="preserve">  side) + packing. Leave a cell blank if the product doesn't use it (e.g. no back</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A UV_TOPCOAT row on a P01 product flags the Mode-B PUV finishing detour.</t>
+          <t xml:space="preserve">  veneer). uv_topcoat_code: fill only if the panel needs a PUV UV-topcoat pass.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Transform_PVS / Transform_PSP: one row per recipe line (kind = INPUT/OUTPUT/STEP).</t>
+          <t>DoorSkin_BOM (PUV Mode-A): board + primer (pass1 + pass2 grams/m²) + packing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Transform_PVS / Transform_PSP: recipe lines (kind = INPUT/OUTPUT/STEP), one row each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>All *_code cells reference codes you defined in the master-data workbook.</t>
         </is>
       </c>
     </row>
@@ -506,21 +521,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,19 +542,19 @@
           <t>★ product_code</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>★ seq</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>★ role</t>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>board_code</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>face_veneer_code</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>back_veneer_code</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
@@ -551,35 +564,25 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>qty</t>
+          <t>face_glue_g</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>usage_g_per_face</t>
+          <t>back_glue_g</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>usage_g_per_m2</t>
+          <t>packing_code</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>qty_unit</t>
+          <t>uv_topcoat_code</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>waste_factor</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>calc_method</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -588,58 +591,48 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DS-OAK-3.2</t>
+          <t>PNL-OAK</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>BRD-MDF-3.2</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>BOARD</t>
+          <t>VNR-OAK-A</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>BRD-MDF-3.2</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
+          <t>VNR-OAK-B</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>GL-STD</t>
+        </is>
+      </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>PER_SHEET</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr"/>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>PKG-CARTON</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"BOARD,FACE_VENEER,BACK_VENEER,FACE_GLUE,BACK_GLUE,PACKING,PRIMER,COATING,UV_TOPCOAT,INPUT,OUTPUT,OTHER"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K3:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PER_SHEET,PER_PALLET"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -650,80 +643,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>★ recipe_code</t>
+          <t>★ product_code</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>★ name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>★ kind</t>
+          <t>★ board_code</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>primer_code</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>seq</t>
+          <t>primer_pass1_g</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>primer_pass2_g</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>packing_code</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>qty</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>uom</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>grade</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>expected_yield_pct</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>expected_loss_pct</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -732,59 +695,37 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>PVS-OAK</t>
+          <t>DS-OAK-3.2</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Oak slicing</t>
+          <t>BRD-MDF-3.2</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>INPUT</t>
+          <t>PRM-UV</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>80</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>OAK-A</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>log</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
+          <t>PKG-CARTON</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"INPUT,OUTPUT,STEP"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -877,6 +818,151 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
+          <t>PVS-OAK</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Oak slicing</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>INPUT</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>OAK-A</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"INPUT,OUTPUT,STEP"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>★ recipe_code</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>★ name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>★ kind</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>seq</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>item_code</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>uom</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>grade</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>expected_yield_pct</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>expected_loss_pct</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
           <t>PSP-OAK</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Data templates: adopt owner's linear Assembly_BOM layout
- Assembly_BOM = owner's exact columns (product_sku, sku_name, pieces_per_unit,
  dims, base_board/face_veneer/face_glue/back_veneer/back_glue code+qty pairs,
  UV_Topcoat_Code + Face/Back Topcoat g/M2, packing_sku_code, Notes). One row per SKU.
- The row also defines the Product, so removed the standalone Product master sheet.
- DoorSkin_BOM (PUV Mode-A primer) kept separate; Transform_PVS/PSP unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/pvwood_bom.xlsx
+++ b/templates/pvwood_bom.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Panel_BOM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Assembly_BOM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DoorSkin_BOM" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Transform_PVS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Transform_PSP" sheetId="5" state="visible" r:id="rId5"/>
@@ -457,35 +457,35 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>★ = required. Fill master data first (items/products/glue recipes must already exist).</t>
+          <t>★ = required. Fill master data first (items / glue recipes must already exist).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ONE ROW PER PRODUCT — fill the component code into each column.</t>
+          <t>ONE ROW PER SKU. The row defines the product (sku_name, pieces_per_unit, dims) AND</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Panel_BOM (main lines P01/P02/P37): board + face/back veneer + glue (g/face each</t>
+          <t>its recipe. Fill each component's code + qty; leave a cell blank if unused (e.g. no</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  side) + packing. Leave a cell blank if the product doesn't use it (e.g. no back</t>
+          <t>back veneer). Glue can differ face vs back (face_glue_code / back_glue_code).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  veneer). uv_topcoat_code: fill only if the panel needs a PUV UV-topcoat pass.</t>
+          <t>UV_Topcoat_Code + Face/Back Topcoat g/M2: fill only if the SKU gets a PUV topcoat.</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>All *_code cells reference codes you defined in the master-data workbook.</t>
+          <t>All *_code / *_sku cells reference codes you defined in the master-data workbook.</t>
         </is>
       </c>
     </row>
@@ -521,70 +521,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>★ product_code</t>
+          <t>★ product_sku</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>board_code</t>
+          <t>sku_name</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>pieces_per_unit</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>thickness_mm</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>width_mm</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>length_mm</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>base_board_code</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>base_board_qty</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>face_veneer_code</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>face_veneer_qty</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>face_glue_code</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>face_glue_qty</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>back_veneer_code</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>glue_recipe_code</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>face_glue_g</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>back_glue_g</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>packing_code</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>uv_topcoat_code</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>back_veneer_qty</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>back_glue_code</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>back_glue_qty</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>UV_Topcoat_Code</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Face_Topcoat_g/M2</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>BackTopcoat_g/M2</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>packing_sku_code</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -596,41 +662,88 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
+          <t>Oak Overlay Panel</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>915</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>2135</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
           <t>BRD-MDF-3.2</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>VNR-OAK-A</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>GL-STD</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>VNR-OAK-B</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>GL-STD</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr"/>
+      <c r="R2" s="4" t="inlineStr"/>
+      <c r="S2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>PKG-CARTON</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
+      <c r="U2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Data templates: unify Assembly_BOM with face/back coating
- Generalize UV_Topcoat -> face/back coating (face_coating_code + Face_Coating_g/M2,
  back_coating_code + Back_Coating_g/M2): serves primer (door skins) OR UV topcoat
  (panels). One Assembly_BOM sheet now covers panels, coated panels, and door skins.
- Removed the separate DoorSkin_BOM sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/pvwood_bom.xlsx
+++ b/templates/pvwood_bom.xlsx
@@ -9,9 +9,8 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Assembly_BOM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DoorSkin_BOM" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Transform_PVS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Transform_PSP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transform_PVS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Transform_PSP" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -485,26 +484,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>UV_Topcoat_Code + Face/Back Topcoat g/M2: fill only if the SKU gets a PUV topcoat.</t>
+          <t>Coating (face/back _coating_code + g/M2) = a primer (door skins) OR a UV topcoat</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DoorSkin_BOM (PUV Mode-A): board + primer (pass1 + pass2 grams/m²) + packing.</t>
+          <t xml:space="preserve">  (panels). Fill only the side(s) that get coated — e.g. a door skin = base board +</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Transform_PVS / Transform_PSP: recipe lines (kind = INPUT/OUTPUT/STEP), one row each.</t>
+          <t xml:space="preserve">  face_coating_code + packing; a UV-topcoat panel = its normal rows + a coating.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Transform_PVS / Transform_PSP: recipe lines (kind = INPUT/OUTPUT/STEP), one row each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>All *_code / *_sku cells reference codes you defined in the master-data workbook.</t>
         </is>
@@ -521,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -540,11 +546,12 @@
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -630,25 +637,30 @@
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
-          <t>UV_Topcoat_Code</t>
+          <t>face_coating_code</t>
         </is>
       </c>
       <c r="R1" s="3" t="inlineStr">
         <is>
-          <t>Face_Topcoat_g/M2</t>
+          <t>Face_Coating_g/M2</t>
         </is>
       </c>
       <c r="S1" s="3" t="inlineStr">
         <is>
-          <t>BackTopcoat_g/M2</t>
+          <t>back_coating_code</t>
         </is>
       </c>
       <c r="T1" s="3" t="inlineStr">
         <is>
+          <t>Back_Coating_g/M2</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
           <t>packing_sku_code</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -738,12 +750,13 @@
       <c r="Q2" s="4" t="inlineStr"/>
       <c r="R2" s="4" t="inlineStr"/>
       <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr"/>
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>PKG-CARTON</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -756,50 +769,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>★ product_code</t>
+          <t>★ recipe_code</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>★ board_code</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>primer_code</t>
+          <t>★ name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>★ kind</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>primer_pass1_g</t>
+          <t>seq</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>primer_pass2_g</t>
+          <t>item_code</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>packing_code</t>
+          <t>role</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>qty</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>uom</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>grade</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>expected_yield_pct</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>expected_loss_pct</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -808,37 +851,59 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DS-OAK-3.2</t>
+          <t>PVS-OAK</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>BRD-MDF-3.2</t>
+          <t>Oak slicing</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>PRM-UV</t>
+          <t>INPUT</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>OAK-A</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>PKG-CARTON</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"INPUT,OUTPUT,STEP"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -931,151 +996,6 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>PVS-OAK</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Oak slicing</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>OAK-A</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>log</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"INPUT,OUTPUT,STEP"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>★ recipe_code</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>★ name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>★ kind</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>seq</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>item_code</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>qty</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>uom</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>grade</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>expected_yield_pct</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>expected_loss_pct</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
           <t>PSP-OAK</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Data templates: drop Species/ProductCategory sheets; product_category on Assembly_BOM
- Remove Species + ProductCategory master sheets. species is now a free-text column
  on Item/Log; the importer auto-masters distinct species + categories (tables kept
  for per-species/per-category reporting).
- Add product_category column to Assembly_BOM (after sku_name).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/pvwood_bom.xlsx
+++ b/templates/pvwood_bom.xlsx
@@ -527,31 +527,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -567,100 +568,105 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>product_category</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>pieces_per_unit</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>thickness_mm</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>width_mm</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>length_mm</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>base_board_code</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>base_board_qty</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>face_veneer_code</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>face_veneer_qty</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>face_glue_code</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>face_glue_qty</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>back_veneer_code</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>back_veneer_qty</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>back_glue_code</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>back_glue_qty</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>face_coating_code</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Face_Coating_g/M2</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>back_coating_code</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Back_Coating_g/M2</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>packing_sku_code</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -679,84 +685,89 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>Overlay Panel</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>300</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>915</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>2135</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>BRD-MDF-3.2</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>VNR-OAK-A</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>GL-STD</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>VNR-OAK-B</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>GL-STD</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr"/>
       <c r="R2" s="4" t="inlineStr"/>
       <c r="S2" s="4" t="inlineStr"/>
       <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>PKG-CARTON</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr"/>
+      <c r="W2" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simplify master data: glue->BOM, logs->Item, drop LogArrival/components
Per owner: trim the master-data workbook to WarehouseLocation/Supplier/Customer/Item.
- Add ItemKind.LOG; a log type is an Item (e.g. LRO4S), each physical log a lot of it
- Drop log / log_arrival / log_document tables (traceability rides on the lot at receiving)
- GlueRecipe sheet moves to the BOM workbook (referenced by face/back_glue_code); glue
  components are just Items (kind=GLUE_COMPONENT) — dropped the GlueRecipe_Components sheet
- Importers updated: master = 4 sheets; import_bom handles GlueRecipe
- Migration applied (fixed drop order); alembic check clean; db ok

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/pvwood_bom.xlsx
+++ b/templates/pvwood_bom.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assembly_BOM" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Transform_PVS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Transform_PSP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GlueRecipe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Assembly_BOM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Transform_PVS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Transform_PSP" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +31,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
     </font>
     <font>
       <b val="1"/>
@@ -65,16 +62,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -456,63 +452,70 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>★ = required. Fill master data first (items / glue recipes must already exist).</t>
+          <t>★ = required. Import master data first (items must exist). GlueRecipe is on its own</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ONE ROW PER SKU. The row defines the product (sku_name, pieces_per_unit, dims) AND</t>
+          <t>sheet here; face/back_glue_code in Assembly_BOM reference these recipe codes.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>its recipe. Fill each component's code + qty; leave a cell blank if unused (e.g. no</t>
+          <t>ONE ROW PER SKU. The row defines the product (sku_name, pieces_per_unit, dims) AND</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>back veneer). Glue can differ face vs back (face_glue_code / back_glue_code).</t>
+          <t>its recipe. Fill each component's code + qty; leave a cell blank if unused (e.g. no</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Coating (face/back _coating_code + g/M2) = a primer (door skins) OR a UV topcoat</t>
+          <t>back veneer). Glue can differ face vs back (face_glue_code / back_glue_code).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (panels). Fill only the side(s) that get coated — e.g. a door skin = base board +</t>
+          <t>Coating (face/back _coating_code + g/M2) = a primer (door skins) OR a UV topcoat</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  face_coating_code + packing; a UV-topcoat panel = its normal rows + a coating.</t>
+          <t xml:space="preserve">  (panels). Fill only the side(s) that get coated.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Transform_PVS / Transform_PSP: recipe lines (kind = INPUT/OUTPUT/STEP), one row each.</t>
+          <t>Transform_PVS / Transform_PSP: recipe lines (kind = INPUT/OUTPUT), one row each —</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>All *_code / *_sku cells reference codes you defined in the master-data workbook.</t>
+          <t xml:space="preserve">  one INPUT (log/veneer) + one OUTPUT per grade. Stages are in the catalog, not here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Item codes reference the master-data Item sheet; glue codes reference GlueRecipe above.</t>
         </is>
       </c>
     </row>
@@ -527,7 +530,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>★ recipe_code</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>★ name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>resin_ratio</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>hardener_ratio</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>extender_ratio</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>filler_ratio</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>water_ratio</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>mix_time_min</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -672,115 +747,18 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>PNL-OAK</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Oak Overlay Panel</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Overlay Panel</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>915</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>2135</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>BRD-MDF-3.2</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>VNR-OAK-A</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>GL-STD</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>VNR-OAK-B</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>GL-STD</t>
-        </is>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>PKG-CARTON</t>
-        </is>
-      </c>
-      <c r="W2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -859,73 +837,23 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>PVS-OAK</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Oak slicing</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>OAK-A</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>log</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"INPUT,OUTPUT,STEP"</formula1>
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"INPUT,OUTPUT"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1004,56 +932,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>PSP-OAK</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Oak splicing</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>INPUT</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>VNR-OAK-CQ-A</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>veneer</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C3:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"INPUT,OUTPUT,STEP"</formula1>
+    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"INPUT,OUTPUT"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>